<commit_message>
Absorb Blind Curator and wire the scored survey into the design
PR #4 added applicability scores but left the one score-10 paper we had
not already cited — The Blind Curator — out of references.md, and left
the spreadsheet orphaned from the design docs.

- Cite Blind Curator as §1.8: false-pass bias silently disables
  contribution-based retirement; contribution is now scored from
  required non-judge criteria only (specs, ADR-0006, architecture).
- Link the scored survey and score-10 bibliographies from README and
  references; list the remaining score-9 papers as next reading.
- Mark Blind Curator cited in the spreadsheet.

Co-authored-by: Rob S <robs@gatech.edu>
</commit_message>
<xml_diff>
--- a/docs/preprints-self-improving-agents.xlsx
+++ b/docs/preprints-self-improving-agents.xlsx
@@ -513,9 +513,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -593,9 +591,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -624,9 +620,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -1101,7 +1095,7 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -11883,7 +11877,6 @@
       <c r="A46" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>Self-Improvements in Modern Agentic Systems (companion survey hub)</t>
@@ -12341,7 +12334,6 @@
       <c r="B11" t="n">
         <v>0</v>
       </c>
-      <c r="C11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>